<commit_message>
Exclude cache artifacts from repository
</commit_message>
<xml_diff>
--- a/batch.xlsx
+++ b/batch.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedroprevost/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedroprevost/ontwikkel/SmartCalc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A50F8B-615C-3449-9AC4-46C5ED31740C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFBB2959-0E82-974C-8150-E3E46B821F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -214,9 +214,6 @@
     <t>6658AL</t>
   </si>
   <si>
-    <t>6658LJ , 6621KW , 6626AP , 6627AC , 6629AX , 6657AT</t>
-  </si>
-  <si>
     <t>6651TG</t>
   </si>
   <si>
@@ -763,9 +760,6 @@
     <t>6657BC</t>
   </si>
   <si>
-    <t>6658XC , 6658DW , 6862BC</t>
-  </si>
-  <si>
     <t>6862XM</t>
   </si>
   <si>
@@ -1052,6 +1046,12 @@
   </si>
   <si>
     <t>Via</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6658LJ , 6621KW , 6657AT, 6626AP , 6627AC , 6629AX </t>
+  </si>
+  <si>
+    <t>6862BC, 6658XC , 6658DW , 6862BC</t>
   </si>
 </sst>
 </file>
@@ -1430,6 +1430,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AE32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="12" max="12" width="55.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -1463,13 +1466,13 @@
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>343</v>
-      </c>
       <c r="M1" s="1" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="N1" t="s">
         <v>10</v>
@@ -1738,17 +1741,17 @@
       <c r="K4" t="s">
         <v>63</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="M4" t="s">
         <v>64</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>65</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>66</v>
-      </c>
-      <c r="O4" t="s">
-        <v>67</v>
       </c>
       <c r="P4">
         <v>6</v>
@@ -1778,33 +1781,33 @@
         <v>62.822666666666997</v>
       </c>
       <c r="Y4" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z4" t="s">
         <v>68</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="AA4" t="s">
         <v>69</v>
       </c>
-      <c r="AA4" t="s">
-        <v>70</v>
-      </c>
       <c r="AB4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AC4" t="s">
         <v>68</v>
       </c>
-      <c r="AC4" t="s">
+      <c r="AD4" t="s">
         <v>69</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D5" t="s">
         <v>58</v>
@@ -1825,19 +1828,19 @@
         <v>61</v>
       </c>
       <c r="J5" t="s">
+        <v>82</v>
+      </c>
+      <c r="K5" t="s">
+        <v>64</v>
+      </c>
+      <c r="M5" t="s">
         <v>83</v>
       </c>
-      <c r="K5" t="s">
+      <c r="N5" t="s">
         <v>65</v>
       </c>
-      <c r="M5" t="s">
+      <c r="O5" t="s">
         <v>84</v>
-      </c>
-      <c r="N5" t="s">
-        <v>66</v>
-      </c>
-      <c r="O5" t="s">
-        <v>85</v>
       </c>
       <c r="P5">
         <v>1</v>
@@ -1867,22 +1870,22 @@
         <v>30.610333333332999</v>
       </c>
       <c r="Y5" t="s">
+        <v>85</v>
+      </c>
+      <c r="Z5" t="s">
         <v>86</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AA5" t="s">
         <v>87</v>
       </c>
-      <c r="AA5" t="s">
-        <v>88</v>
-      </c>
       <c r="AB5" t="s">
+        <v>85</v>
+      </c>
+      <c r="AC5" t="s">
         <v>86</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AD5" t="s">
         <v>87</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.2">
@@ -1890,10 +1893,10 @@
         <v>56</v>
       </c>
       <c r="B6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D6" t="s">
         <v>58</v>
@@ -1905,7 +1908,7 @@
         <v>32</v>
       </c>
       <c r="G6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H6">
         <v>397</v>
@@ -1914,19 +1917,19 @@
         <v>34</v>
       </c>
       <c r="J6" t="s">
+        <v>91</v>
+      </c>
+      <c r="K6" t="s">
         <v>92</v>
       </c>
-      <c r="K6" t="s">
+      <c r="M6" t="s">
         <v>93</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>94</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>95</v>
-      </c>
-      <c r="O6" t="s">
-        <v>96</v>
       </c>
       <c r="P6">
         <v>1</v>
@@ -1956,22 +1959,22 @@
         <v>25.110666666667001</v>
       </c>
       <c r="Y6" t="s">
+        <v>96</v>
+      </c>
+      <c r="Z6" t="s">
         <v>97</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AA6" t="s">
         <v>98</v>
       </c>
-      <c r="AA6" t="s">
-        <v>99</v>
-      </c>
       <c r="AB6" t="s">
+        <v>96</v>
+      </c>
+      <c r="AC6" t="s">
         <v>97</v>
       </c>
-      <c r="AC6" t="s">
+      <c r="AD6" t="s">
         <v>98</v>
-      </c>
-      <c r="AD6" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.2">
@@ -1979,10 +1982,10 @@
         <v>56</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D7" t="s">
         <v>58</v>
@@ -1994,7 +1997,7 @@
         <v>32</v>
       </c>
       <c r="G7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H7">
         <v>309</v>
@@ -2003,22 +2006,22 @@
         <v>61</v>
       </c>
       <c r="J7" t="s">
+        <v>102</v>
+      </c>
+      <c r="K7" t="s">
+        <v>93</v>
+      </c>
+      <c r="L7" t="s">
         <v>103</v>
       </c>
-      <c r="K7" t="s">
-        <v>94</v>
-      </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>104</v>
-      </c>
-      <c r="M7" t="s">
-        <v>105</v>
       </c>
       <c r="N7" t="s">
         <v>38</v>
       </c>
       <c r="O7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P7">
         <v>6</v>
@@ -2048,22 +2051,22 @@
         <v>70.679333333333005</v>
       </c>
       <c r="Y7" t="s">
+        <v>106</v>
+      </c>
+      <c r="Z7" t="s">
         <v>107</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="AA7" t="s">
         <v>108</v>
       </c>
-      <c r="AA7" t="s">
-        <v>109</v>
-      </c>
       <c r="AB7" t="s">
+        <v>106</v>
+      </c>
+      <c r="AC7" t="s">
         <v>107</v>
       </c>
-      <c r="AC7" t="s">
+      <c r="AD7" t="s">
         <v>108</v>
-      </c>
-      <c r="AD7" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.2">
@@ -2071,10 +2074,10 @@
         <v>56</v>
       </c>
       <c r="B8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D8" t="s">
         <v>58</v>
@@ -2095,19 +2098,19 @@
         <v>61</v>
       </c>
       <c r="J8" t="s">
+        <v>110</v>
+      </c>
+      <c r="K8" t="s">
         <v>111</v>
       </c>
-      <c r="K8" t="s">
+      <c r="M8" t="s">
         <v>112</v>
       </c>
-      <c r="M8" t="s">
+      <c r="N8" t="s">
         <v>113</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>114</v>
-      </c>
-      <c r="O8" t="s">
-        <v>115</v>
       </c>
       <c r="P8">
         <v>1</v>
@@ -2137,22 +2140,22 @@
         <v>22.753666666667002</v>
       </c>
       <c r="Y8" t="s">
+        <v>115</v>
+      </c>
+      <c r="Z8" t="s">
         <v>116</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="AA8" t="s">
         <v>117</v>
       </c>
-      <c r="AA8" t="s">
-        <v>118</v>
-      </c>
       <c r="AB8" t="s">
+        <v>115</v>
+      </c>
+      <c r="AC8" t="s">
         <v>116</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AD8" t="s">
         <v>117</v>
-      </c>
-      <c r="AD8" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.2">
@@ -2160,10 +2163,10 @@
         <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D9" t="s">
         <v>58</v>
@@ -2184,22 +2187,22 @@
         <v>45</v>
       </c>
       <c r="J9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K9" t="s">
         <v>37</v>
       </c>
       <c r="L9" t="s">
+        <v>123</v>
+      </c>
+      <c r="M9" t="s">
         <v>124</v>
       </c>
-      <c r="M9" t="s">
+      <c r="N9" t="s">
         <v>125</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>126</v>
-      </c>
-      <c r="O9" t="s">
-        <v>127</v>
       </c>
       <c r="P9">
         <v>4</v>
@@ -2229,22 +2232,22 @@
         <v>57.630666666666997</v>
       </c>
       <c r="Y9" t="s">
+        <v>127</v>
+      </c>
+      <c r="Z9" t="s">
         <v>128</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="AA9" t="s">
         <v>129</v>
       </c>
-      <c r="AA9" t="s">
+      <c r="AB9" t="s">
         <v>130</v>
       </c>
-      <c r="AB9" t="s">
+      <c r="AC9" t="s">
         <v>131</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="AD9" t="s">
         <v>132</v>
-      </c>
-      <c r="AD9" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.2">
@@ -2252,10 +2255,10 @@
         <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D10" t="s">
         <v>58</v>
@@ -2267,7 +2270,7 @@
         <v>32</v>
       </c>
       <c r="G10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H10">
         <v>391</v>
@@ -2276,19 +2279,19 @@
         <v>34</v>
       </c>
       <c r="J10" t="s">
+        <v>136</v>
+      </c>
+      <c r="K10" t="s">
         <v>137</v>
       </c>
-      <c r="K10" t="s">
-        <v>138</v>
-      </c>
       <c r="M10" t="s">
+        <v>124</v>
+      </c>
+      <c r="N10" t="s">
         <v>125</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>126</v>
-      </c>
-      <c r="O10" t="s">
-        <v>127</v>
       </c>
       <c r="P10">
         <v>1</v>
@@ -2318,22 +2321,22 @@
         <v>27.467666666667</v>
       </c>
       <c r="Y10" t="s">
+        <v>138</v>
+      </c>
+      <c r="Z10" t="s">
         <v>139</v>
       </c>
-      <c r="Z10" t="s">
+      <c r="AA10" t="s">
         <v>140</v>
       </c>
-      <c r="AA10" t="s">
-        <v>141</v>
-      </c>
       <c r="AB10" t="s">
+        <v>138</v>
+      </c>
+      <c r="AC10" t="s">
         <v>139</v>
       </c>
-      <c r="AC10" t="s">
+      <c r="AD10" t="s">
         <v>140</v>
-      </c>
-      <c r="AD10" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.2">
@@ -2341,10 +2344,10 @@
         <v>56</v>
       </c>
       <c r="B11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D11" t="s">
         <v>58</v>
@@ -2356,31 +2359,31 @@
         <v>32</v>
       </c>
       <c r="G11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H11">
         <v>17</v>
       </c>
       <c r="I11" t="s">
+        <v>144</v>
+      </c>
+      <c r="J11" t="s">
         <v>145</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>146</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>147</v>
       </c>
-      <c r="L11" t="s">
-        <v>148</v>
-      </c>
       <c r="M11" t="s">
+        <v>124</v>
+      </c>
+      <c r="N11" t="s">
         <v>125</v>
       </c>
-      <c r="N11" t="s">
-        <v>126</v>
-      </c>
       <c r="O11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P11">
         <v>27</v>
@@ -2407,22 +2410,22 @@
         <v>187.11199999999999</v>
       </c>
       <c r="Y11" t="s">
+        <v>148</v>
+      </c>
+      <c r="Z11" t="s">
         <v>149</v>
       </c>
-      <c r="Z11" t="s">
+      <c r="AA11" t="s">
         <v>150</v>
       </c>
-      <c r="AA11" t="s">
-        <v>151</v>
-      </c>
       <c r="AB11" t="s">
+        <v>148</v>
+      </c>
+      <c r="AC11" t="s">
         <v>149</v>
       </c>
-      <c r="AC11" t="s">
+      <c r="AD11" t="s">
         <v>150</v>
-      </c>
-      <c r="AD11" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.2">
@@ -2430,10 +2433,10 @@
         <v>56</v>
       </c>
       <c r="B12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D12" t="s">
         <v>58</v>
@@ -2445,7 +2448,7 @@
         <v>32</v>
       </c>
       <c r="G12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H12">
         <v>391</v>
@@ -2454,19 +2457,19 @@
         <v>34</v>
       </c>
       <c r="J12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K12" t="s">
         <v>153</v>
       </c>
-      <c r="K12" t="s">
+      <c r="M12" t="s">
         <v>154</v>
       </c>
-      <c r="M12" t="s">
+      <c r="N12" t="s">
         <v>155</v>
       </c>
-      <c r="N12" t="s">
-        <v>156</v>
-      </c>
       <c r="O12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="P12">
         <v>1</v>
@@ -2496,22 +2499,22 @@
         <v>36.288666666666998</v>
       </c>
       <c r="Y12" t="s">
+        <v>156</v>
+      </c>
+      <c r="Z12" t="s">
         <v>157</v>
       </c>
-      <c r="Z12" t="s">
+      <c r="AA12" t="s">
         <v>158</v>
       </c>
-      <c r="AA12" t="s">
-        <v>159</v>
-      </c>
       <c r="AB12" t="s">
+        <v>156</v>
+      </c>
+      <c r="AC12" t="s">
         <v>157</v>
       </c>
-      <c r="AC12" t="s">
+      <c r="AD12" t="s">
         <v>158</v>
-      </c>
-      <c r="AD12" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
@@ -2519,10 +2522,10 @@
         <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D13" t="s">
         <v>58</v>
@@ -2534,7 +2537,7 @@
         <v>32</v>
       </c>
       <c r="G13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H13">
         <v>411</v>
@@ -2543,19 +2546,19 @@
         <v>34</v>
       </c>
       <c r="J13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K13" t="s">
         <v>162</v>
       </c>
-      <c r="K13" t="s">
+      <c r="M13" t="s">
         <v>163</v>
       </c>
-      <c r="M13" t="s">
+      <c r="N13" t="s">
         <v>164</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>165</v>
-      </c>
-      <c r="O13" t="s">
-        <v>166</v>
       </c>
       <c r="P13">
         <v>1</v>
@@ -2585,22 +2588,22 @@
         <v>45.618499999999997</v>
       </c>
       <c r="Y13" t="s">
+        <v>166</v>
+      </c>
+      <c r="Z13" t="s">
         <v>167</v>
       </c>
-      <c r="Z13" t="s">
+      <c r="AA13" t="s">
         <v>168</v>
       </c>
-      <c r="AA13" t="s">
-        <v>169</v>
-      </c>
       <c r="AB13" t="s">
+        <v>166</v>
+      </c>
+      <c r="AC13" t="s">
         <v>167</v>
       </c>
-      <c r="AC13" t="s">
+      <c r="AD13" t="s">
         <v>168</v>
-      </c>
-      <c r="AD13" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
@@ -2608,10 +2611,10 @@
         <v>56</v>
       </c>
       <c r="B14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D14" t="s">
         <v>58</v>
@@ -2623,7 +2626,7 @@
         <v>32</v>
       </c>
       <c r="G14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H14">
         <v>290</v>
@@ -2632,22 +2635,22 @@
         <v>61</v>
       </c>
       <c r="J14" t="s">
+        <v>171</v>
+      </c>
+      <c r="K14" t="s">
         <v>172</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>173</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>174</v>
       </c>
-      <c r="M14" t="s">
+      <c r="N14" t="s">
         <v>175</v>
       </c>
-      <c r="N14" t="s">
+      <c r="O14" t="s">
         <v>176</v>
-      </c>
-      <c r="O14" t="s">
-        <v>177</v>
       </c>
       <c r="P14">
         <v>3</v>
@@ -2677,22 +2680,22 @@
         <v>62.581833333333002</v>
       </c>
       <c r="Y14" t="s">
+        <v>177</v>
+      </c>
+      <c r="Z14" t="s">
         <v>178</v>
       </c>
-      <c r="Z14" t="s">
+      <c r="AA14" t="s">
         <v>179</v>
       </c>
-      <c r="AA14" t="s">
-        <v>180</v>
-      </c>
       <c r="AB14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC14" t="s">
         <v>178</v>
       </c>
-      <c r="AC14" t="s">
+      <c r="AD14" t="s">
         <v>179</v>
-      </c>
-      <c r="AD14" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.2">
@@ -2700,10 +2703,10 @@
         <v>56</v>
       </c>
       <c r="B15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D15" t="s">
         <v>58</v>
@@ -2715,7 +2718,7 @@
         <v>32</v>
       </c>
       <c r="G15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H15">
         <v>308</v>
@@ -2724,22 +2727,22 @@
         <v>61</v>
       </c>
       <c r="J15" t="s">
+        <v>182</v>
+      </c>
+      <c r="K15" t="s">
         <v>183</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>184</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>185</v>
       </c>
-      <c r="M15" t="s">
+      <c r="N15" t="s">
         <v>186</v>
       </c>
-      <c r="N15" t="s">
-        <v>187</v>
-      </c>
       <c r="O15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P15">
         <v>6</v>
@@ -2769,22 +2772,22 @@
         <v>69.367166666667003</v>
       </c>
       <c r="Y15" t="s">
+        <v>187</v>
+      </c>
+      <c r="Z15" t="s">
         <v>188</v>
       </c>
-      <c r="Z15" t="s">
+      <c r="AA15" t="s">
         <v>189</v>
       </c>
-      <c r="AA15" t="s">
-        <v>190</v>
-      </c>
       <c r="AB15" t="s">
+        <v>187</v>
+      </c>
+      <c r="AC15" t="s">
         <v>188</v>
       </c>
-      <c r="AC15" t="s">
+      <c r="AD15" t="s">
         <v>189</v>
-      </c>
-      <c r="AD15" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.2">
@@ -2792,10 +2795,10 @@
         <v>56</v>
       </c>
       <c r="B16" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C16" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D16" t="s">
         <v>58</v>
@@ -2807,7 +2810,7 @@
         <v>32</v>
       </c>
       <c r="G16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H16">
         <v>1952</v>
@@ -2816,22 +2819,22 @@
         <v>34</v>
       </c>
       <c r="J16" t="s">
+        <v>192</v>
+      </c>
+      <c r="K16" t="s">
         <v>193</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>194</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>195</v>
       </c>
-      <c r="M16" t="s">
+      <c r="N16" t="s">
         <v>196</v>
       </c>
-      <c r="N16" t="s">
+      <c r="O16" t="s">
         <v>197</v>
-      </c>
-      <c r="O16" t="s">
-        <v>198</v>
       </c>
       <c r="P16">
         <v>3</v>
@@ -2861,22 +2864,22 @@
         <v>65.126333333332994</v>
       </c>
       <c r="Y16" t="s">
+        <v>198</v>
+      </c>
+      <c r="Z16" t="s">
         <v>199</v>
       </c>
-      <c r="Z16" t="s">
+      <c r="AA16" t="s">
         <v>200</v>
       </c>
-      <c r="AA16" t="s">
-        <v>201</v>
-      </c>
       <c r="AB16" t="s">
+        <v>198</v>
+      </c>
+      <c r="AC16" t="s">
         <v>199</v>
       </c>
-      <c r="AC16" t="s">
+      <c r="AD16" t="s">
         <v>200</v>
-      </c>
-      <c r="AD16" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="17" spans="1:30" x14ac:dyDescent="0.2">
@@ -2884,10 +2887,10 @@
         <v>56</v>
       </c>
       <c r="B17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D17" t="s">
         <v>58</v>
@@ -2899,7 +2902,7 @@
         <v>32</v>
       </c>
       <c r="G17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H17">
         <v>2057</v>
@@ -2908,22 +2911,22 @@
         <v>34</v>
       </c>
       <c r="J17" t="s">
+        <v>203</v>
+      </c>
+      <c r="K17" t="s">
         <v>204</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>205</v>
       </c>
-      <c r="L17" t="s">
+      <c r="M17" t="s">
         <v>206</v>
       </c>
-      <c r="M17" t="s">
-        <v>207</v>
-      </c>
       <c r="N17" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O17" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P17">
         <v>4</v>
@@ -2953,36 +2956,36 @@
         <v>78.697000000000003</v>
       </c>
       <c r="Y17" t="s">
+        <v>207</v>
+      </c>
+      <c r="Z17" t="s">
         <v>208</v>
       </c>
-      <c r="Z17" t="s">
+      <c r="AA17" t="s">
         <v>209</v>
       </c>
-      <c r="AA17" t="s">
-        <v>210</v>
-      </c>
       <c r="AB17" t="s">
+        <v>207</v>
+      </c>
+      <c r="AC17" t="s">
         <v>208</v>
       </c>
-      <c r="AC17" t="s">
+      <c r="AD17" t="s">
         <v>209</v>
-      </c>
-      <c r="AD17" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" t="s">
+        <v>210</v>
+      </c>
+      <c r="C18" t="s">
+        <v>210</v>
+      </c>
+      <c r="D18" t="s">
         <v>73</v>
-      </c>
-      <c r="B18" t="s">
-        <v>211</v>
-      </c>
-      <c r="C18" t="s">
-        <v>211</v>
-      </c>
-      <c r="D18" t="s">
-        <v>74</v>
       </c>
       <c r="E18" t="s">
         <v>59</v>
@@ -2991,7 +2994,7 @@
         <v>32</v>
       </c>
       <c r="G18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H18">
         <v>2057</v>
@@ -3000,19 +3003,19 @@
         <v>61</v>
       </c>
       <c r="J18" t="s">
+        <v>211</v>
+      </c>
+      <c r="K18" t="s">
         <v>212</v>
       </c>
-      <c r="K18" t="s">
+      <c r="M18" t="s">
+        <v>206</v>
+      </c>
+      <c r="N18" t="s">
+        <v>180</v>
+      </c>
+      <c r="O18" t="s">
         <v>213</v>
-      </c>
-      <c r="M18" t="s">
-        <v>207</v>
-      </c>
-      <c r="N18" t="s">
-        <v>181</v>
-      </c>
-      <c r="O18" t="s">
-        <v>214</v>
       </c>
       <c r="P18">
         <v>1</v>
@@ -3042,36 +3045,36 @@
         <v>42.225833333333</v>
       </c>
       <c r="Y18" t="s">
+        <v>214</v>
+      </c>
+      <c r="Z18" t="s">
         <v>215</v>
       </c>
-      <c r="Z18" t="s">
+      <c r="AA18" t="s">
         <v>216</v>
       </c>
-      <c r="AA18" t="s">
-        <v>217</v>
-      </c>
       <c r="AB18" t="s">
+        <v>214</v>
+      </c>
+      <c r="AC18" t="s">
         <v>215</v>
       </c>
-      <c r="AC18" t="s">
+      <c r="AD18" t="s">
         <v>216</v>
-      </c>
-      <c r="AD18" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" t="s">
+        <v>217</v>
+      </c>
+      <c r="C19" t="s">
+        <v>217</v>
+      </c>
+      <c r="D19" t="s">
         <v>73</v>
-      </c>
-      <c r="B19" t="s">
-        <v>218</v>
-      </c>
-      <c r="C19" t="s">
-        <v>218</v>
-      </c>
-      <c r="D19" t="s">
-        <v>74</v>
       </c>
       <c r="E19" t="s">
         <v>59</v>
@@ -3080,7 +3083,7 @@
         <v>32</v>
       </c>
       <c r="G19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H19">
         <v>288</v>
@@ -3089,19 +3092,19 @@
         <v>61</v>
       </c>
       <c r="J19" t="s">
+        <v>218</v>
+      </c>
+      <c r="K19" t="s">
         <v>219</v>
       </c>
-      <c r="K19" t="s">
+      <c r="M19" t="s">
+        <v>185</v>
+      </c>
+      <c r="N19" t="s">
         <v>220</v>
       </c>
-      <c r="M19" t="s">
-        <v>186</v>
-      </c>
-      <c r="N19" t="s">
-        <v>221</v>
-      </c>
       <c r="O19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P19">
         <v>1</v>
@@ -3131,22 +3134,22 @@
         <v>38.833166666666997</v>
       </c>
       <c r="Y19" t="s">
+        <v>221</v>
+      </c>
+      <c r="Z19" t="s">
         <v>222</v>
       </c>
-      <c r="Z19" t="s">
+      <c r="AA19" t="s">
         <v>223</v>
       </c>
-      <c r="AA19" t="s">
-        <v>224</v>
-      </c>
       <c r="AB19" t="s">
+        <v>221</v>
+      </c>
+      <c r="AC19" t="s">
         <v>222</v>
       </c>
-      <c r="AC19" t="s">
+      <c r="AD19" t="s">
         <v>223</v>
-      </c>
-      <c r="AD19" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.2">
@@ -3154,10 +3157,10 @@
         <v>56</v>
       </c>
       <c r="B20" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C20" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D20" t="s">
         <v>58</v>
@@ -3169,7 +3172,7 @@
         <v>32</v>
       </c>
       <c r="G20" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H20">
         <v>395</v>
@@ -3178,22 +3181,22 @@
         <v>61</v>
       </c>
       <c r="J20" t="s">
+        <v>226</v>
+      </c>
+      <c r="K20" t="s">
         <v>227</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>228</v>
       </c>
-      <c r="L20" t="s">
+      <c r="M20" t="s">
         <v>229</v>
       </c>
-      <c r="M20" t="s">
+      <c r="N20" t="s">
         <v>230</v>
       </c>
-      <c r="N20" t="s">
-        <v>231</v>
-      </c>
       <c r="O20" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P20">
         <v>3</v>
@@ -3223,22 +3226,22 @@
         <v>67.670833333332993</v>
       </c>
       <c r="Y20" t="s">
+        <v>231</v>
+      </c>
+      <c r="Z20" t="s">
         <v>232</v>
       </c>
-      <c r="Z20" t="s">
+      <c r="AA20" t="s">
         <v>233</v>
       </c>
-      <c r="AA20" t="s">
-        <v>234</v>
-      </c>
       <c r="AB20" t="s">
+        <v>231</v>
+      </c>
+      <c r="AC20" t="s">
         <v>232</v>
       </c>
-      <c r="AC20" t="s">
+      <c r="AD20" t="s">
         <v>233</v>
-      </c>
-      <c r="AD20" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.2">
@@ -3246,10 +3249,10 @@
         <v>56</v>
       </c>
       <c r="B21" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C21" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D21" t="s">
         <v>58</v>
@@ -3261,7 +3264,7 @@
         <v>32</v>
       </c>
       <c r="G21" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H21">
         <v>1792</v>
@@ -3270,19 +3273,19 @@
         <v>34</v>
       </c>
       <c r="J21" t="s">
+        <v>235</v>
+      </c>
+      <c r="K21" t="s">
         <v>236</v>
       </c>
-      <c r="K21" t="s">
+      <c r="M21" t="s">
         <v>237</v>
       </c>
-      <c r="M21" t="s">
+      <c r="N21" t="s">
         <v>238</v>
       </c>
-      <c r="N21" t="s">
+      <c r="O21" t="s">
         <v>239</v>
-      </c>
-      <c r="O21" t="s">
-        <v>240</v>
       </c>
       <c r="P21">
         <v>1</v>
@@ -3312,22 +3315,22 @@
         <v>43.073999999999998</v>
       </c>
       <c r="Y21" t="s">
+        <v>240</v>
+      </c>
+      <c r="Z21" t="s">
         <v>241</v>
       </c>
-      <c r="Z21" t="s">
+      <c r="AA21" t="s">
         <v>242</v>
       </c>
-      <c r="AA21" t="s">
-        <v>243</v>
-      </c>
       <c r="AB21" t="s">
+        <v>240</v>
+      </c>
+      <c r="AC21" t="s">
         <v>241</v>
       </c>
-      <c r="AC21" t="s">
+      <c r="AD21" t="s">
         <v>242</v>
-      </c>
-      <c r="AD21" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="22" spans="1:30" x14ac:dyDescent="0.2">
@@ -3335,10 +3338,10 @@
         <v>56</v>
       </c>
       <c r="B22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D22" t="s">
         <v>58</v>
@@ -3350,7 +3353,7 @@
         <v>32</v>
       </c>
       <c r="G22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H22">
         <v>2191</v>
@@ -3359,22 +3362,22 @@
         <v>61</v>
       </c>
       <c r="J22" t="s">
+        <v>244</v>
+      </c>
+      <c r="K22" t="s">
         <v>245</v>
       </c>
-      <c r="K22" t="s">
+      <c r="L22" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="M22" t="s">
         <v>246</v>
       </c>
-      <c r="L22" t="s">
+      <c r="N22" t="s">
         <v>247</v>
       </c>
-      <c r="M22" t="s">
-        <v>248</v>
-      </c>
-      <c r="N22" t="s">
-        <v>249</v>
-      </c>
       <c r="O22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P22">
         <v>3</v>
@@ -3404,22 +3407,22 @@
         <v>55.796500000000002</v>
       </c>
       <c r="Y22" t="s">
+        <v>248</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>249</v>
+      </c>
+      <c r="AA22" t="s">
         <v>250</v>
       </c>
-      <c r="Z22" t="s">
-        <v>251</v>
-      </c>
-      <c r="AA22" t="s">
-        <v>252</v>
-      </c>
       <c r="AB22" t="s">
+        <v>248</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>249</v>
+      </c>
+      <c r="AD22" t="s">
         <v>250</v>
-      </c>
-      <c r="AC22" t="s">
-        <v>251</v>
-      </c>
-      <c r="AD22" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="23" spans="1:30" x14ac:dyDescent="0.2">
@@ -3427,10 +3430,10 @@
         <v>56</v>
       </c>
       <c r="B23" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C23" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D23" t="s">
         <v>58</v>
@@ -3442,7 +3445,7 @@
         <v>32</v>
       </c>
       <c r="G23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H23">
         <v>401</v>
@@ -3451,22 +3454,22 @@
         <v>61</v>
       </c>
       <c r="J23" t="s">
+        <v>252</v>
+      </c>
+      <c r="K23" t="s">
+        <v>253</v>
+      </c>
+      <c r="L23" t="s">
         <v>254</v>
       </c>
-      <c r="K23" t="s">
+      <c r="M23" t="s">
         <v>255</v>
       </c>
-      <c r="L23" t="s">
+      <c r="N23" t="s">
         <v>256</v>
       </c>
-      <c r="M23" t="s">
-        <v>257</v>
-      </c>
-      <c r="N23" t="s">
-        <v>258</v>
-      </c>
       <c r="O23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P23">
         <v>4</v>
@@ -3496,22 +3499,22 @@
         <v>54.948333333332997</v>
       </c>
       <c r="Y23" t="s">
+        <v>257</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>258</v>
+      </c>
+      <c r="AA23" t="s">
         <v>259</v>
       </c>
-      <c r="Z23" t="s">
-        <v>260</v>
-      </c>
-      <c r="AA23" t="s">
-        <v>261</v>
-      </c>
       <c r="AB23" t="s">
+        <v>257</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>258</v>
+      </c>
+      <c r="AD23" t="s">
         <v>259</v>
-      </c>
-      <c r="AC23" t="s">
-        <v>260</v>
-      </c>
-      <c r="AD23" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.2">
@@ -3519,10 +3522,10 @@
         <v>56</v>
       </c>
       <c r="B24" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C24" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D24" t="s">
         <v>58</v>
@@ -3534,7 +3537,7 @@
         <v>32</v>
       </c>
       <c r="G24" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H24">
         <v>2075</v>
@@ -3543,22 +3546,22 @@
         <v>34</v>
       </c>
       <c r="J24" t="s">
+        <v>262</v>
+      </c>
+      <c r="K24" t="s">
+        <v>263</v>
+      </c>
+      <c r="L24" t="s">
+        <v>260</v>
+      </c>
+      <c r="M24" t="s">
+        <v>253</v>
+      </c>
+      <c r="N24" t="s">
         <v>264</v>
       </c>
-      <c r="K24" t="s">
-        <v>265</v>
-      </c>
-      <c r="L24" t="s">
-        <v>262</v>
-      </c>
-      <c r="M24" t="s">
-        <v>255</v>
-      </c>
-      <c r="N24" t="s">
-        <v>266</v>
-      </c>
       <c r="O24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P24">
         <v>2</v>
@@ -3588,22 +3591,22 @@
         <v>48.162999999999997</v>
       </c>
       <c r="Y24" t="s">
+        <v>265</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>266</v>
+      </c>
+      <c r="AA24" t="s">
         <v>267</v>
       </c>
-      <c r="Z24" t="s">
-        <v>268</v>
-      </c>
-      <c r="AA24" t="s">
-        <v>269</v>
-      </c>
       <c r="AB24" t="s">
+        <v>265</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>266</v>
+      </c>
+      <c r="AD24" t="s">
         <v>267</v>
-      </c>
-      <c r="AC24" t="s">
-        <v>268</v>
-      </c>
-      <c r="AD24" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="25" spans="1:30" x14ac:dyDescent="0.2">
@@ -3611,10 +3614,10 @@
         <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C25" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D25" t="s">
         <v>58</v>
@@ -3626,7 +3629,7 @@
         <v>32</v>
       </c>
       <c r="G25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H25">
         <v>316</v>
@@ -3635,22 +3638,22 @@
         <v>45</v>
       </c>
       <c r="J25" t="s">
+        <v>270</v>
+      </c>
+      <c r="K25" t="s">
+        <v>271</v>
+      </c>
+      <c r="L25" t="s">
         <v>272</v>
       </c>
-      <c r="K25" t="s">
+      <c r="M25" t="s">
         <v>273</v>
       </c>
-      <c r="L25" t="s">
+      <c r="N25" t="s">
         <v>274</v>
       </c>
-      <c r="M25" t="s">
-        <v>275</v>
-      </c>
-      <c r="N25" t="s">
-        <v>276</v>
-      </c>
       <c r="O25" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P25">
         <v>5</v>
@@ -3680,22 +3683,22 @@
         <v>60.8855</v>
       </c>
       <c r="Y25" t="s">
+        <v>275</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>276</v>
+      </c>
+      <c r="AA25" t="s">
         <v>277</v>
       </c>
-      <c r="Z25" t="s">
-        <v>278</v>
-      </c>
-      <c r="AA25" t="s">
-        <v>279</v>
-      </c>
       <c r="AB25" t="s">
+        <v>275</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>276</v>
+      </c>
+      <c r="AD25" t="s">
         <v>277</v>
-      </c>
-      <c r="AC25" t="s">
-        <v>278</v>
-      </c>
-      <c r="AD25" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="26" spans="1:30" x14ac:dyDescent="0.2">
@@ -3703,10 +3706,10 @@
         <v>56</v>
       </c>
       <c r="B26" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C26" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D26" t="s">
         <v>58</v>
@@ -3718,7 +3721,7 @@
         <v>32</v>
       </c>
       <c r="G26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H26">
         <v>410</v>
@@ -3727,22 +3730,22 @@
         <v>61</v>
       </c>
       <c r="J26" t="s">
+        <v>279</v>
+      </c>
+      <c r="K26" t="s">
+        <v>280</v>
+      </c>
+      <c r="L26" t="s">
         <v>281</v>
       </c>
-      <c r="K26" t="s">
+      <c r="M26" t="s">
         <v>282</v>
       </c>
-      <c r="L26" t="s">
+      <c r="N26" t="s">
         <v>283</v>
       </c>
-      <c r="M26" t="s">
-        <v>284</v>
-      </c>
-      <c r="N26" t="s">
-        <v>285</v>
-      </c>
       <c r="O26" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P26">
         <v>6</v>
@@ -3772,22 +3775,22 @@
         <v>58.341000000000001</v>
       </c>
       <c r="Y26" t="s">
+        <v>284</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>285</v>
+      </c>
+      <c r="AA26" t="s">
         <v>286</v>
       </c>
-      <c r="Z26" t="s">
+      <c r="AB26" t="s">
         <v>287</v>
       </c>
-      <c r="AA26" t="s">
+      <c r="AC26" t="s">
         <v>288</v>
       </c>
-      <c r="AB26" t="s">
+      <c r="AD26" t="s">
         <v>289</v>
-      </c>
-      <c r="AC26" t="s">
-        <v>290</v>
-      </c>
-      <c r="AD26" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="27" spans="1:30" x14ac:dyDescent="0.2">
@@ -3795,10 +3798,10 @@
         <v>56</v>
       </c>
       <c r="B27" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C27" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D27" t="s">
         <v>58</v>
@@ -3810,7 +3813,7 @@
         <v>32</v>
       </c>
       <c r="G27" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H27">
         <v>2075</v>
@@ -3819,19 +3822,19 @@
         <v>61</v>
       </c>
       <c r="J27" t="s">
+        <v>291</v>
+      </c>
+      <c r="K27" t="s">
+        <v>292</v>
+      </c>
+      <c r="M27" t="s">
         <v>293</v>
       </c>
-      <c r="K27" t="s">
+      <c r="N27" t="s">
         <v>294</v>
       </c>
-      <c r="M27" t="s">
-        <v>295</v>
-      </c>
-      <c r="N27" t="s">
-        <v>296</v>
-      </c>
       <c r="O27" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P27">
         <v>1</v>
@@ -3861,22 +3864,22 @@
         <v>32.896000000000001</v>
       </c>
       <c r="Y27" t="s">
+        <v>295</v>
+      </c>
+      <c r="Z27" t="s">
+        <v>296</v>
+      </c>
+      <c r="AA27" t="s">
         <v>297</v>
       </c>
-      <c r="Z27" t="s">
-        <v>298</v>
-      </c>
-      <c r="AA27" t="s">
-        <v>299</v>
-      </c>
       <c r="AB27" t="s">
+        <v>295</v>
+      </c>
+      <c r="AC27" t="s">
+        <v>296</v>
+      </c>
+      <c r="AD27" t="s">
         <v>297</v>
-      </c>
-      <c r="AC27" t="s">
-        <v>298</v>
-      </c>
-      <c r="AD27" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.2">
@@ -3884,10 +3887,10 @@
         <v>56</v>
       </c>
       <c r="B28" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C28" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D28" t="s">
         <v>58</v>
@@ -3899,7 +3902,7 @@
         <v>32</v>
       </c>
       <c r="G28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H28">
         <v>2057</v>
@@ -3908,19 +3911,19 @@
         <v>61</v>
       </c>
       <c r="J28" t="s">
+        <v>299</v>
+      </c>
+      <c r="K28" t="s">
+        <v>300</v>
+      </c>
+      <c r="M28" t="s">
         <v>301</v>
       </c>
-      <c r="K28" t="s">
+      <c r="N28" t="s">
         <v>302</v>
       </c>
-      <c r="M28" t="s">
-        <v>303</v>
-      </c>
-      <c r="N28" t="s">
-        <v>304</v>
-      </c>
       <c r="O28" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="P28">
         <v>1</v>
@@ -3950,36 +3953,36 @@
         <v>35.4405</v>
       </c>
       <c r="Y28" t="s">
+        <v>303</v>
+      </c>
+      <c r="Z28" t="s">
+        <v>304</v>
+      </c>
+      <c r="AA28" t="s">
         <v>305</v>
       </c>
-      <c r="Z28" t="s">
-        <v>306</v>
-      </c>
-      <c r="AA28" t="s">
-        <v>307</v>
-      </c>
       <c r="AB28" t="s">
+        <v>303</v>
+      </c>
+      <c r="AC28" t="s">
+        <v>304</v>
+      </c>
+      <c r="AD28" t="s">
         <v>305</v>
-      </c>
-      <c r="AC28" t="s">
-        <v>306</v>
-      </c>
-      <c r="AD28" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="29" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>74</v>
+      </c>
+      <c r="B29" t="s">
+        <v>306</v>
+      </c>
+      <c r="C29" t="s">
+        <v>306</v>
+      </c>
+      <c r="D29" t="s">
         <v>75</v>
-      </c>
-      <c r="B29" t="s">
-        <v>308</v>
-      </c>
-      <c r="C29" t="s">
-        <v>308</v>
-      </c>
-      <c r="D29" t="s">
-        <v>76</v>
       </c>
       <c r="E29" t="s">
         <v>31</v>
@@ -3988,7 +3991,7 @@
         <v>32</v>
       </c>
       <c r="G29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H29">
         <v>2191</v>
@@ -3997,19 +4000,19 @@
         <v>34</v>
       </c>
       <c r="J29" t="s">
+        <v>307</v>
+      </c>
+      <c r="K29" t="s">
+        <v>308</v>
+      </c>
+      <c r="M29" t="s">
         <v>309</v>
       </c>
-      <c r="K29" t="s">
+      <c r="N29" t="s">
         <v>310</v>
       </c>
-      <c r="M29" t="s">
-        <v>311</v>
-      </c>
-      <c r="N29" t="s">
-        <v>312</v>
-      </c>
       <c r="O29" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="P29">
         <v>1</v>
@@ -4039,22 +4042,22 @@
         <v>34.592333333333002</v>
       </c>
       <c r="Y29" t="s">
+        <v>311</v>
+      </c>
+      <c r="Z29" t="s">
+        <v>312</v>
+      </c>
+      <c r="AA29" t="s">
         <v>313</v>
       </c>
-      <c r="Z29" t="s">
-        <v>314</v>
-      </c>
-      <c r="AA29" t="s">
-        <v>315</v>
-      </c>
       <c r="AB29" t="s">
+        <v>311</v>
+      </c>
+      <c r="AC29" t="s">
+        <v>312</v>
+      </c>
+      <c r="AD29" t="s">
         <v>313</v>
-      </c>
-      <c r="AC29" t="s">
-        <v>314</v>
-      </c>
-      <c r="AD29" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="30" spans="1:30" x14ac:dyDescent="0.2">
@@ -4062,10 +4065,10 @@
         <v>56</v>
       </c>
       <c r="B30" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C30" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D30" t="s">
         <v>58</v>
@@ -4077,7 +4080,7 @@
         <v>32</v>
       </c>
       <c r="G30" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H30">
         <v>1670</v>
@@ -4086,22 +4089,22 @@
         <v>34</v>
       </c>
       <c r="J30" t="s">
+        <v>315</v>
+      </c>
+      <c r="K30" t="s">
+        <v>309</v>
+      </c>
+      <c r="L30" t="s">
+        <v>316</v>
+      </c>
+      <c r="M30" t="s">
         <v>317</v>
       </c>
-      <c r="K30" t="s">
-        <v>311</v>
-      </c>
-      <c r="L30" t="s">
+      <c r="N30" t="s">
         <v>318</v>
       </c>
-      <c r="M30" t="s">
-        <v>319</v>
-      </c>
-      <c r="N30" t="s">
-        <v>320</v>
-      </c>
       <c r="O30" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P30">
         <v>2</v>
@@ -4131,22 +4134,22 @@
         <v>56.644666666667</v>
       </c>
       <c r="Y30" t="s">
+        <v>319</v>
+      </c>
+      <c r="Z30" t="s">
+        <v>320</v>
+      </c>
+      <c r="AA30" t="s">
         <v>321</v>
       </c>
-      <c r="Z30" t="s">
-        <v>322</v>
-      </c>
-      <c r="AA30" t="s">
-        <v>323</v>
-      </c>
       <c r="AB30" t="s">
+        <v>319</v>
+      </c>
+      <c r="AC30" t="s">
+        <v>320</v>
+      </c>
+      <c r="AD30" t="s">
         <v>321</v>
-      </c>
-      <c r="AC30" t="s">
-        <v>322</v>
-      </c>
-      <c r="AD30" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="31" spans="1:30" x14ac:dyDescent="0.2">
@@ -4154,10 +4157,10 @@
         <v>56</v>
       </c>
       <c r="B31" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C31" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D31" t="s">
         <v>58</v>
@@ -4169,7 +4172,7 @@
         <v>32</v>
       </c>
       <c r="G31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H31">
         <v>1920</v>
@@ -4178,22 +4181,22 @@
         <v>34</v>
       </c>
       <c r="J31" t="s">
+        <v>323</v>
+      </c>
+      <c r="K31" t="s">
+        <v>324</v>
+      </c>
+      <c r="L31" t="s">
         <v>325</v>
       </c>
-      <c r="K31" t="s">
+      <c r="M31" t="s">
         <v>326</v>
       </c>
-      <c r="L31" t="s">
+      <c r="N31" t="s">
         <v>327</v>
       </c>
-      <c r="M31" t="s">
-        <v>328</v>
-      </c>
-      <c r="N31" t="s">
-        <v>329</v>
-      </c>
       <c r="O31" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P31">
         <v>2</v>
@@ -4223,22 +4226,22 @@
         <v>60.037333333333002</v>
       </c>
       <c r="Y31" t="s">
+        <v>328</v>
+      </c>
+      <c r="Z31" t="s">
+        <v>329</v>
+      </c>
+      <c r="AA31" t="s">
         <v>330</v>
       </c>
-      <c r="Z31" t="s">
-        <v>331</v>
-      </c>
-      <c r="AA31" t="s">
-        <v>332</v>
-      </c>
       <c r="AB31" t="s">
+        <v>328</v>
+      </c>
+      <c r="AC31" t="s">
+        <v>329</v>
+      </c>
+      <c r="AD31" t="s">
         <v>330</v>
-      </c>
-      <c r="AC31" t="s">
-        <v>331</v>
-      </c>
-      <c r="AD31" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="32" spans="1:30" x14ac:dyDescent="0.2">
@@ -4246,10 +4249,10 @@
         <v>56</v>
       </c>
       <c r="B32" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C32" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D32" t="s">
         <v>58</v>
@@ -4261,7 +4264,7 @@
         <v>32</v>
       </c>
       <c r="G32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H32">
         <v>322</v>
@@ -4270,22 +4273,22 @@
         <v>61</v>
       </c>
       <c r="J32" t="s">
+        <v>332</v>
+      </c>
+      <c r="K32" t="s">
+        <v>333</v>
+      </c>
+      <c r="L32" t="s">
         <v>334</v>
       </c>
-      <c r="K32" t="s">
+      <c r="M32" t="s">
         <v>335</v>
       </c>
-      <c r="L32" t="s">
-        <v>336</v>
-      </c>
-      <c r="M32" t="s">
-        <v>337</v>
-      </c>
       <c r="N32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O32" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="P32">
         <v>2</v>
@@ -4315,22 +4318,22 @@
         <v>23.539333333333001</v>
       </c>
       <c r="Y32" t="s">
+        <v>336</v>
+      </c>
+      <c r="Z32" t="s">
+        <v>337</v>
+      </c>
+      <c r="AA32" t="s">
         <v>338</v>
       </c>
-      <c r="Z32" t="s">
-        <v>339</v>
-      </c>
-      <c r="AA32" t="s">
-        <v>340</v>
-      </c>
       <c r="AB32" t="s">
+        <v>336</v>
+      </c>
+      <c r="AC32" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD32" t="s">
         <v>338</v>
-      </c>
-      <c r="AC32" t="s">
-        <v>339</v>
-      </c>
-      <c r="AD32" t="s">
-        <v>340</v>
       </c>
     </row>
   </sheetData>

</xml_diff>